<commit_message>
결과 파일 업데이트 2026-08-13 10:15
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260813.xlsx
+++ b/results/andar_할인율모니터링_20260813.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H175"/>
+  <dimension ref="A1:H176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7,196</t>
+          <t>7,198</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>275</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>275</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>275</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>577</t>
+          <t>578</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9,938</t>
+          <t>9,939</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>320</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>441</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>1,059</t>
+          <t>1,060</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10,279</t>
+          <t>10,280</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>1,932</t>
+          <t>1,933</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>6,474</t>
+          <t>6,475</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>222</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>628</t>
+          <t>629</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>196</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>3,133</t>
+          <t>3,134</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>3,133</t>
+          <t>3,134</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>731</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>70</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>171</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>476</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>476</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>171</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>552</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>635</t>
+          <t>636</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>537</t>
+          <t>538</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>327</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>1,932</t>
+          <t>1,933</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6119,7 +6119,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -7673,7 +7673,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>552</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -7685,82 +7685,124 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11092&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ENTSO-03</t>
+          <t>ENTSC-05</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>안다르 이지무브 화이트</t>
+          <t>에어프레시 크루 삭스</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>129,000</t>
+          <t>17,000</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>64,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>496</t>
+          <t>575</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>ENTSO-03</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>안다르 이지무브 화이트</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>129,000</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>64,500</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>496</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
           <t>https://andar.co.kr/product/detail.html?product_no=12512&amp;cate_no=2111&amp;display_group=1</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B176" t="inlineStr">
         <is>
           <t>ENTSO-03</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C176" t="inlineStr">
         <is>
           <t>안다르 이지무브 베이지</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr">
+      <c r="D176" t="inlineStr">
         <is>
           <t>129,000</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr">
+      <c r="E176" t="inlineStr">
         <is>
           <t>64,500</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F176" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
+      <c r="G176" t="inlineStr">
         <is>
           <t>414</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
+      <c r="H176" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>

</xml_diff>